<commit_message>
feat: very high push allows a very risky trade at the nearest end of diversion (very_risky_eod); graph, mind maps, workbook, docs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ltp-trading-rules.xlsx
+++ b/docs/ltp-trading-rules.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Conditions'!$A$1:$E$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pressure pairs'!$A$1:$M$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All cases'!$A$1:$S$530</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rules'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rules'!$A$1:$D$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -588,7 +588,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Tug of war (owner rule): a risky trade is allowed when both sides push the same way, or one pushes highly and the other is stable. Bears winning = risky short, bulls winning = risky long, at the level the live tool shows as Risky. Sides pulling against each other are contested: no risky trade. Decide from the outcome, not from the first-level scenario number.</t>
+          <t>Tug of war (owner rule): a risky trade is allowed when both sides push the same way, or one pushes highly and the other is stable. Bears winning = risky short, bulls winning = risky long, at the level the live tool shows as Risky. Very high push (both the same way, at least one high): a very risky trade at the nearest end of diversion. Sides pulling against each other are contested: no risky trade. Decide from the outcome, not from the first-level scenario number.</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr"/>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S34" s="3" t="inlineStr">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="R47" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S47" s="3" t="inlineStr">
@@ -8749,7 +8749,7 @@
       </c>
       <c r="R59" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S59" s="3" t="inlineStr">
@@ -9568,7 +9568,7 @@
       </c>
       <c r="R68" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S68" s="3" t="inlineStr">
@@ -9841,7 +9841,7 @@
       </c>
       <c r="R71" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S71" s="3" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="R72" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S72" s="3" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="R76" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S76" s="3" t="inlineStr">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="R77" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S77" s="3" t="inlineStr">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="R78" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S78" s="3" t="inlineStr">
@@ -10842,7 +10842,7 @@
       </c>
       <c r="R82" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S82" s="3" t="inlineStr">
@@ -10933,7 +10933,7 @@
       </c>
       <c r="R83" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S83" s="3" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="R86" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S86" s="3" t="inlineStr">
@@ -11297,7 +11297,7 @@
       </c>
       <c r="R87" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S87" s="3" t="inlineStr">
@@ -11388,7 +11388,7 @@
       </c>
       <c r="R88" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S88" s="3" t="inlineStr">
@@ -11752,7 +11752,7 @@
       </c>
       <c r="R92" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S92" s="3" t="inlineStr">
@@ -12389,7 +12389,7 @@
       </c>
       <c r="R99" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S99" s="3" t="inlineStr">
@@ -13572,7 +13572,7 @@
       </c>
       <c r="R112" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S112" s="3" t="inlineStr">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="R124" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S124" s="3" t="inlineStr">
@@ -15847,7 +15847,7 @@
       </c>
       <c r="R137" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S137" s="3" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="R150" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S150" s="3" t="inlineStr">
@@ -18304,7 +18304,7 @@
       </c>
       <c r="R164" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S164" s="3" t="inlineStr">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="R177" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S177" s="3" t="inlineStr">
@@ -20852,7 +20852,7 @@
       </c>
       <c r="R192" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S192" s="3" t="inlineStr">
@@ -21216,7 +21216,7 @@
       </c>
       <c r="R196" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S196" s="3" t="inlineStr">
@@ -21307,7 +21307,7 @@
       </c>
       <c r="R197" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S197" s="3" t="inlineStr">
@@ -21489,7 +21489,7 @@
       </c>
       <c r="R199" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S199" s="3" t="inlineStr">
@@ -21580,7 +21580,7 @@
       </c>
       <c r="R200" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S200" s="3" t="inlineStr">
@@ -21853,7 +21853,7 @@
       </c>
       <c r="R203" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S203" s="3" t="inlineStr">
@@ -23127,7 +23127,7 @@
       </c>
       <c r="R217" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S217" s="3" t="inlineStr">
@@ -23582,7 +23582,7 @@
       </c>
       <c r="R222" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S222" s="3" t="inlineStr">
@@ -24037,7 +24037,7 @@
       </c>
       <c r="R227" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S227" s="3" t="inlineStr">
@@ -25857,7 +25857,7 @@
       </c>
       <c r="R247" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S247" s="3" t="inlineStr">
@@ -26312,7 +26312,7 @@
       </c>
       <c r="R252" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S252" s="3" t="inlineStr">
@@ -27313,7 +27313,7 @@
       </c>
       <c r="R263" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S263" s="3" t="inlineStr">
@@ -27586,7 +27586,7 @@
       </c>
       <c r="R266" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S266" s="3" t="inlineStr">
@@ -27677,7 +27677,7 @@
       </c>
       <c r="R267" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S267" s="3" t="inlineStr">
@@ -27859,7 +27859,7 @@
       </c>
       <c r="R269" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S269" s="3" t="inlineStr">
@@ -27950,7 +27950,7 @@
       </c>
       <c r="R270" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S270" s="3" t="inlineStr">
@@ -28132,7 +28132,7 @@
       </c>
       <c r="R272" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S272" s="3" t="inlineStr">
@@ -28587,7 +28587,7 @@
       </c>
       <c r="R277" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S277" s="3" t="inlineStr">
@@ -30407,7 +30407,7 @@
       </c>
       <c r="R297" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S297" s="3" t="inlineStr">
@@ -31226,7 +31226,7 @@
       </c>
       <c r="R306" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S306" s="3" t="inlineStr">
@@ -32045,7 +32045,7 @@
       </c>
       <c r="R315" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S315" s="3" t="inlineStr">
@@ -32318,7 +32318,7 @@
       </c>
       <c r="R318" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S318" s="3" t="inlineStr">
@@ -32409,7 +32409,7 @@
       </c>
       <c r="R319" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S319" s="3" t="inlineStr">
@@ -32773,7 +32773,7 @@
       </c>
       <c r="R323" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S323" s="3" t="inlineStr">
@@ -32864,7 +32864,7 @@
       </c>
       <c r="R324" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S324" s="3" t="inlineStr">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="R325" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S325" s="3" t="inlineStr">
@@ -33683,7 +33683,7 @@
       </c>
       <c r="R333" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S333" s="3" t="inlineStr">
@@ -34775,7 +34775,7 @@
       </c>
       <c r="R345" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S345" s="3" t="inlineStr">
@@ -35958,7 +35958,7 @@
       </c>
       <c r="R358" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S358" s="3" t="inlineStr">
@@ -37232,7 +37232,7 @@
       </c>
       <c r="R372" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S372" s="3" t="inlineStr">
@@ -38051,7 +38051,7 @@
       </c>
       <c r="R381" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S381" s="3" t="inlineStr">
@@ -38142,7 +38142,7 @@
       </c>
       <c r="R382" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S382" s="3" t="inlineStr">
@@ -38415,7 +38415,7 @@
       </c>
       <c r="R385" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S385" s="3" t="inlineStr">
@@ -38506,7 +38506,7 @@
       </c>
       <c r="R386" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S386" s="3" t="inlineStr">
@@ -38597,7 +38597,7 @@
       </c>
       <c r="R387" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S387" s="3" t="inlineStr">
@@ -38961,7 +38961,7 @@
       </c>
       <c r="R391" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S391" s="3" t="inlineStr">
@@ -39507,7 +39507,7 @@
       </c>
       <c r="R397" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S397" s="3" t="inlineStr">
@@ -40781,7 +40781,7 @@
       </c>
       <c r="R411" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S411" s="3" t="inlineStr">
@@ -41964,7 +41964,7 @@
       </c>
       <c r="R424" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S424" s="3" t="inlineStr">
@@ -42692,7 +42692,7 @@
       </c>
       <c r="R432" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S432" s="3" t="inlineStr">
@@ -43056,7 +43056,7 @@
       </c>
       <c r="R436" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S436" s="3" t="inlineStr">
@@ -43147,7 +43147,7 @@
       </c>
       <c r="R437" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S437" s="3" t="inlineStr">
@@ -43329,7 +43329,7 @@
       </c>
       <c r="R439" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S439" s="3" t="inlineStr">
@@ -43420,7 +43420,7 @@
       </c>
       <c r="R440" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S440" s="3" t="inlineStr">
@@ -44057,7 +44057,7 @@
       </c>
       <c r="R447" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S447" s="3" t="inlineStr">
@@ -44512,7 +44512,7 @@
       </c>
       <c r="R452" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S452" s="3" t="inlineStr">
@@ -44967,7 +44967,7 @@
       </c>
       <c r="R457" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S457" s="3" t="inlineStr">
@@ -45331,7 +45331,7 @@
       </c>
       <c r="R461" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S461" s="3" t="inlineStr">
@@ -45422,7 +45422,7 @@
       </c>
       <c r="R462" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S462" s="3" t="inlineStr">
@@ -45604,7 +45604,7 @@
       </c>
       <c r="R464" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S464" s="3" t="inlineStr">
@@ -45695,7 +45695,7 @@
       </c>
       <c r="R465" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S465" s="3" t="inlineStr">
@@ -46332,7 +46332,7 @@
       </c>
       <c r="R472" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S472" s="3" t="inlineStr">
@@ -46787,7 +46787,7 @@
       </c>
       <c r="R477" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S477" s="3" t="inlineStr">
@@ -47788,7 +47788,7 @@
       </c>
       <c r="R488" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S488" s="3" t="inlineStr">
@@ -48152,7 +48152,7 @@
       </c>
       <c r="R492" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S492" s="3" t="inlineStr">
@@ -50063,7 +50063,7 @@
       </c>
       <c r="R513" s="3" t="inlineStr">
         <is>
-          <t>Risky LONG allowed at the tool's Risky level</t>
+          <t>VERY RISKY LONG allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S513" s="3" t="inlineStr">
@@ -50427,7 +50427,7 @@
       </c>
       <c r="R517" s="3" t="inlineStr">
         <is>
-          <t>Risky SHORT allowed at the tool's Risky level</t>
+          <t>VERY RISKY SHORT allowed at the nearest end of diversion (and a risky one at the tool's Risky level)</t>
         </is>
       </c>
       <c r="S517" s="3" t="inlineStr">
@@ -51631,7 +51631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -51797,27 +51797,49 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Very high push allows very risky trades at the nearest end of diversion (EOD)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Very high = both sides push the same way and at least one pushes highly (highly with plain, or both highly). Bears winning: a very risky short at the nearest end of diversion above the price; bulls winning: a very risky long at the nearest end of diversion below it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>The live tool shows the risky and moderate levels itself</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Use the tool's displayed Risky and Moderate values, not our own formula (ours, EOR-1 / EOS+1, was a guess).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: regenerate workbook with the one-diversion stop rule
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ltp-trading-rules.xlsx
+++ b/docs/ltp-trading-rules.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Conditions'!$A$1:$E$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pressure pairs'!$A$1:$M$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All cases'!$A$1:$S$530</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rules'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rules'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -594,6 +594,13 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Stop loss (owner rule): every trade risks exactly one diversion, one strike step from the entry: 50 points in NIFTY, 100 in BANKNIFTY and SENSEX, for every setup. The agent has it as v2.0 stop_rule one_diversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>The pressure of each condition is our reading of the tool's wording, confirmed with the owner condition by condition on 2026-10-13. "~" in the app means the history is not one of the listed shapes.</t>
         </is>
@@ -51631,7 +51638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -51797,7 +51804,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Very high push allows very risky trades at the nearest end of diversion (EOD)</t>
+          <t>Every trade risks one diversion: the stop is one strike step from the entry (NIFTY 50 points, BANKNIFTY and SENSEX 100)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -51812,34 +51819,56 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Very high = both sides push the same way and at least one pushes highly (highly with plain, or both highly). Bears winning: a very risky short at the nearest end of diversion above the price; bulls winning: a very risky long at the nearest end of diversion below it.</t>
+          <t>Applies to every setup in v2.0 (reversal, 9:20, SOC, risky, very risky). Earlier versions keep the 9:20 style stop.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Very high push allows very risky trades at the nearest end of diversion (EOD)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Very high = both sides push the same way and at least one pushes highly (highly with plain, or both highly). Bears winning: a very risky short at the nearest end of diversion above the price; bulls winning: a very risky long at the nearest end of diversion below it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>The live tool shows the risky and moderate levels itself</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Use the tool's displayed Risky and Moderate values, not our own formula (ours, EOR-1 / EOS+1, was a guess).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>